<commit_message>
feat: implements sample reuse
</commit_message>
<xml_diff>
--- a/experiments/reports/experiments.xlsx
+++ b/experiments/reports/experiments.xlsx
@@ -14,11 +14,11 @@
     <sheet name="Predictions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Experiments'!$A$1:$AE$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stages'!$A$1:$J$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Artifacts'!$A$1:$H$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Evaluations'!$A$1:$D$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Predictions'!$A$1:$F$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Experiments'!$A$1:$AE$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stages'!$A$1:$J$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Artifacts'!$A$1:$H$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Evaluations'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Predictions'!$A$1:$F$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -849,8 +849,141 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CSOP TDS baseline</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>LightGBM prediction of TDS for candidate subgraphs.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.907977Z</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.921989Z</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:16.081190Z</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>integration_test_graph</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>data/raw/graph_test</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>networkx_random_paths</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O4" t="n">
+        <v>42</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>graph-size-and-local-degree-v1</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>["num_vertices","num_edges","degree_mean","degree_max","degree_min","degree_std"]</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>tds</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="U4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="W4" t="n">
+        <v>42</v>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>lightgbm</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>{"learning_rate":0.1,"min_child_samples":1,"n_estimators":5,"num_leaves":5,"random_state":42,"verbosity":-1}</t>
+        </is>
+      </c>
+      <c r="Z4" t="n">
+        <v>0.159201</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>189202432</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>{"mae":0.09841499819109839,"r2":0.5641519743660988,"rmse":0.11003131191139048}</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/config/experiment.json</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/environment/environment.json</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AE3"/>
+  <autoFilter ref="A1:AE4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -861,7 +994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1504,8 +1637,302 @@
         <v>4096</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>36</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>graph_loading</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.925339Z</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.937943Z</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>0.01258194399997592</v>
+      </c>
+      <c r="H16" t="n">
+        <v>183128064</v>
+      </c>
+      <c r="I16" t="n">
+        <v>183140352</v>
+      </c>
+      <c r="J16" t="n">
+        <v>12288</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>37</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>dataset_construction</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.941055Z</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.976407Z</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>0.03533265800069785</v>
+      </c>
+      <c r="H17" t="n">
+        <v>183140352</v>
+      </c>
+      <c r="I17" t="n">
+        <v>184717312</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1576960</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>38</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>dataset_loading</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.979533Z</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.986176Z</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>0.006611615001020255</v>
+      </c>
+      <c r="H18" t="n">
+        <v>184717312</v>
+      </c>
+      <c r="I18" t="n">
+        <v>184950784</v>
+      </c>
+      <c r="J18" t="n">
+        <v>233472</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>39</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>train_test_split</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.989083Z</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.994805Z</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>0.005706940002710326</v>
+      </c>
+      <c r="H19" t="n">
+        <v>184950784</v>
+      </c>
+      <c r="I19" t="n">
+        <v>185004032</v>
+      </c>
+      <c r="J19" t="n">
+        <v>53248</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>40</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>split_dataset_persistence</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.997776Z</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:16.011056Z</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>0.01326458499897853</v>
+      </c>
+      <c r="H20" t="n">
+        <v>185004032</v>
+      </c>
+      <c r="I20" t="n">
+        <v>185024512</v>
+      </c>
+      <c r="J20" t="n">
+        <v>20480</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>41</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>model_training</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:16.013998Z</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:16.050472Z</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>0.03645643100026064</v>
+      </c>
+      <c r="H21" t="n">
+        <v>185024512</v>
+      </c>
+      <c r="I21" t="n">
+        <v>189198336</v>
+      </c>
+      <c r="J21" t="n">
+        <v>4173824</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>42</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>test_prediction_and_evaluation</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:16.053560Z</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:16.064113Z</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>0.01053614400007064</v>
+      </c>
+      <c r="H22" t="n">
+        <v>189198336</v>
+      </c>
+      <c r="I22" t="n">
+        <v>189202432</v>
+      </c>
+      <c r="J22" t="n">
+        <v>4096</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J15"/>
+  <autoFilter ref="A1:J22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1516,7 +1943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3001,8 +3428,728 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe:config</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>experiment.json</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/config/experiment.json</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>1138</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.913896Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe:environment</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>environment</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>environment.json</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/environment/environment.json</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>559</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.918775Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ART_38b7bc87b9454d7c8ebb9b57f418eb0b</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>graphs</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>metadata</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>text/plain</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/graphs/integration_test_graph/metadata</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>3</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.927355Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ART_f11926029f8545b18ba3108d56cbbb30</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>graphs</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>adjlist</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>text/plain</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/graphs/integration_test_graph/adjlist</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>47</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.931246Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ART_9a02de10e5df422ebb1ecfd976701214</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>graphs</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>metadata.json</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/graphs/integration_test_graph/metadata.json</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>163</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.934863Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ART_d57a3f8e6551499086e33a9c208b95bb</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>subgraphs</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>subgraph_000000.json</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/subgraphs/integration_test_graph/subgraph_000000.json</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>144</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.945041Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ART_c96e27aa6c234dbe8ead357b82f99fc1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>subgraphs</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>subgraph_000001.json</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/subgraphs/integration_test_graph/subgraph_000001.json</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>211</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.949036Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ART_4e91012cc25f4f27a016f021e24c0852</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>subgraphs</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>subgraph_000002.json</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/subgraphs/integration_test_graph/subgraph_000002.json</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>144</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.952484Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ART_64a8c546339d4529b05b2aac96b64388</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>subgraphs</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>subgraph_000003.json</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/subgraphs/integration_test_graph/subgraph_000003.json</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>211</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.956000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ART_e3ecad565e634b2eb0c89faa12552e61</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>subgraphs</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>subgraph_000004.json</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/subgraphs/integration_test_graph/subgraph_000004.json</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>181</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.959505Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ART_5860c5cf8640489fafb1b7451198c1af</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>subgraphs</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>subgraph_000005.json</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/subgraphs/integration_test_graph/subgraph_000005.json</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>144</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.962904Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ART_514775ebf52f47869dda3aea1d062508</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>datasets</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>dataset.csv</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>text/csv</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/datasets/dataset.csv</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>426</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.983082Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ART_32cb2a23292a484fba9d16e64554cf0d</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>datasets</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>train_dataset.csv</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>text/csv</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/datasets/train_dataset.csv</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>321</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:15.999877Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ART_26e07215510a4ab6b0f1669e04baac16</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>datasets</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>test_dataset.csv</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>text/csv</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/datasets/test_dataset.csv</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>201</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:16.004527Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ART_6a7f7c53963b45e2813481ca4ef8b97a</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>datasets</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>split_metadata.json</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/datasets/split_metadata.json</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>185</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:16.008010Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ART_5d4e95eb47704e578647686646174362</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>models</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>lightgbm_model.txt</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>text/plain</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/models/lightgbm_model.txt</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>4967</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:16.046841Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ART_271b20a36b824dea98fffc2756502c8f</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>predictions</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>predictions.csv</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>text/csv</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/predictions/predictions.csv</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>281</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:16.057408Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ART_f32f68d2a22c4e769ffee417684d4e67</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>evaluation</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>metrics.json</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>experiments/runs/EXP_20261008_35c87eb4a7fe/evaluation/metrics.json</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>137</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:19:16.061042Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H37"/>
+  <autoFilter ref="A1:H55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3013,7 +4160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3146,8 +4293,62 @@
         <v>0.5641519743660988</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.09841499819109839</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>17</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>rmse</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.1100313119113905</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>18</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.5641519743660988</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D7"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3158,7 +4359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3289,8 +4490,56 @@
         <v>-0.147622494896253</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>11</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>integration_test_graph:0</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.04920750148594381</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.04920750148594381</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EXP_20261008_35c87eb4a7fe</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>12</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>integration_test_graph:1</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.1857108384370803</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-0.147622494896253</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F5"/>
+  <autoFilter ref="A1:F7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>